<commit_message>
Updates thematicanalysis reference and adds archimate model
</commit_message>
<xml_diff>
--- a/Thematic Analysis.xlsx
+++ b/Thematic Analysis.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="175">
   <si>
     <t>Theme ID</t>
   </si>
@@ -45,7 +45,7 @@
     <t>Complex and variable healthcare BPMN models</t>
   </si>
   <si>
-    <t>Modelling and Analysis of Complex Patient-Treatment Process Using GraphMiner Toolbox</t>
+    <t>Metsker, O., Kesarev, S., Bolgova, E., Golubev, K., Karsakov, A., Yakovlev, A., &amp; Kovalchuk, S. (2019). Modelling and analysis of complex patient-treatment process using GraphMiner Toolbox. In J. M. F. Rodrigues, P. J. S. Cardoso, J. Monteiro, R. Lam, V. V. Krzhizhanovskaya, M. H. Lees, J. J. Dongarra, &amp; P. M. A. Sloot (Eds.), Computational science—ICCS 2019 (pp. 674–680). Springer International Publishing.</t>
   </si>
   <si>
     <t>"The results were poorly interpreted because the process map was characterized by variability and high complexity"</t>
@@ -81,7 +81,19 @@
     <t>High variability and complexity of process maps</t>
   </si>
   <si>
-    <t>Efficient Discovery of Compact Maximal Behavioral Patterns from Event Logs</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Acheli, M., Grigori, D., &amp; Weidlich, M. (2019). Efficient discovery of compact maximal behavioral patterns from event logs. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/978-3-030-21290-2_36</t>
+    </r>
   </si>
   <si>
     <t>"The reason being that there is a large variability of the behavior of different process instances and a model capturing all variations tends to be complex"</t>
@@ -90,7 +102,19 @@
     <t>Difficulty extracting actionable insights from variable healthcare models</t>
   </si>
   <si>
-    <t>Mining and exploring care pathways from electronic medical records with visual analytics</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Perer, A., Wang, F., &amp; Hu, J. (2015). Mining and exploring care pathways from electronic medical records with visual analytics. Journal of Biomedical Informatics, 56, 369–378. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1016/j.jbi.2015.06.020</t>
+    </r>
   </si>
   <si>
     <t>“Applying BPM techniques to real patient data [...] results in very complex and chaotic graphs.”</t>
@@ -105,7 +129,19 @@
     <t>Manual effort for parameters</t>
   </si>
   <si>
-    <t>Big Data Analytics in Healthcare: Data-Driven Methods for Typical Treatment Pattern Mining</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Guo, C., &amp; Chen, J. (2019). Big data analytics in healthcare: Data-driven methods for typical treatment pattern mining. Journal of Systems Science and Systems Engineering, 28(6), 694–714. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s11518-019-5437-5</t>
+    </r>
   </si>
   <si>
     <t>“Firstly, due to the complex and varying-length of treatment records, the fixed intervals of treatment periods maybe not the optimal split. Secondly, in experimental setting, some parameters need to be manually defined aforehand, such as the weights of different treatment periods, the threshold of typical drugs, the definition of the core area for a treatment cluster, and so on.”</t>
@@ -123,7 +159,7 @@
     <t>Discovery</t>
   </si>
   <si>
-    <t>Crowd-Based Mining of Reusable Process Model Patterns</t>
+    <t>Rodríguez, C., Daniel, F., &amp; Casati, F. (2014). Crowd-based mining of reusable process model patterns. In S. Sadiq, P. Soffer, &amp; H. Völzer (Eds.), Business process management (pp. 51–66). Springer International Publishing.</t>
   </si>
   <si>
     <t>“The approach however suffers from problems that are common to pattern mining algorithms: identifying support threshold values, managing large numbers of produced patterns, coping with noise (useless patterns), giving meaning to patterns, and the cold start problem. Inspired by the recent advent of crowdsourcing, the intuition emerged that it might be possible to attack these problems with the help of the crowd, that is, by involving humans in the mining process.”</t>
@@ -132,7 +168,19 @@
     <t>Difficulty configuring thresholds</t>
   </si>
   <si>
-    <t>Comparative Analysis of Frequent Pattern Mining Algorithms on Healthcare Data</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Jhanjhi, N. Z. (2024). Comparative analysis of frequent pattern mining algorithms on healthcare data. In 2024 IEEE 9th International Conference on Engineering Technologies and Applied Sciences (ICETAS) (pp. 1–10). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/ICETAS62372.2024.11119839</t>
+    </r>
   </si>
   <si>
     <t>“This analysis involved varying the minimum support values and observing their impact on the number of frequent itemsets generated and the execution time required to compute them. This approach provides valuable insights into how the minimum support parameter influences both the quantity of discovered patterns and the computational load.”</t>
@@ -141,7 +189,19 @@
     <t>Parameter sensitivity of minimum support threshold tuning makes it efficient for better insight extraction</t>
   </si>
   <si>
-    <t>Opportunities and challenges for applying process mining in healthcare: a systematic mapping study</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Dallagassa, M. R., dos Santos Garcia, C., Scalabrin, E. E., Ioshii, S. O., &amp; Carvalho, D. R. (2022). Opportunities and challenges for applying process mining in healthcare: A systematic mapping study. Journal of Ambient Intelligence and Humanized Computing, 13(1), 165–182. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s12652-021-02894-7</t>
+    </r>
   </si>
   <si>
     <t>“The approaches presented often deal with analyses geared towards a specific context, a pathology or a surgical procedure, which require time in the definition of parameters and expert knowledge of the Health field.”</t>
@@ -156,6 +216,9 @@
     <t>Domain and modelling knowledge gap</t>
   </si>
   <si>
+    <t>Guo, C., &amp; Chen, J. (2019). Big data analytics in healthcare: Data-driven methods for typical treatment pattern mining. Journal of Systems Science and Systems Engineering, 28(6), 694–714. https://doi.org/10.1007/s11518-019-5437-5</t>
+  </si>
+  <si>
     <t>“Before their use, patterns were checked by a mashup expert assuring their meaningfulness and reusability. The intuition stems from the observation that pure statistical support does not always imply interestingness, and that human experts are anyway the ultimate responsibles for deciding about the suitability or not of patterns.”</t>
   </si>
   <si>
@@ -177,7 +240,19 @@
     <t>Analysts need healthcare context / domain knowledge</t>
   </si>
   <si>
-    <t>Sequential Pattern Mining of Electronic Healthcare Reimbursement Claims: Experiences and Challenges in Uncovering How Patients are Treated by Physicians</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Malhotra, K., Hobson, T. C., Valkova, S., Pullum, L. L., &amp; Ramanathan, A. (2015). Sequential pattern mining of electronic healthcare reimbursement claims: Experiences and challenges in uncovering how patients are treated by physicians. In 2015 IEEE International Conference on Big Data (Big Data) (pp. 2670–2679). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/BigData.2015.7364067</t>
+    </r>
   </si>
   <si>
     <t>“Integrating such clinically relevant parameters [...] and extracting meaningful results will be critical for advancing data-driven decision making.”</t>
@@ -192,6 +267,21 @@
     <t>Scalability and time-critical mining limitations</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Jhanjhi, N. Z. (2024). Comparative analysis of frequent pattern mining algorithms on healthcare data. In 2024 IEEE 9th International Conference on Engineering Technologies and Applied Sciences (ICETAS) (pp. 1–10). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/ICETAS62372.2024.11119839</t>
+    </r>
+  </si>
+  <si>
     <t>“Our analysis focused on the number of frequent itemsets generated and the execution time for each algorithm, revealing significant differences in efficiency and effectiveness. This analysis involved varying the minimum support values and observing their impact on the number of frequent itemsets generated and the execution time required to compute them. This approach provides valuable insights into how the minimum support parameter influences both the quantity of discovered patterns and the computational load.”</t>
   </si>
   <si>
@@ -204,7 +294,19 @@
     <t>AI-enhanced pattern mining system should estimate the expected mining time before executing pattern discovery, so that users can make informed decisions about whether to proceed, adjust parameters, increase/reduce dataset or postpone the operation based on time constraints.</t>
   </si>
   <si>
-    <t>Process Mining in Cardiology: A Literature Review</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Kusuma, G. P., Hall, M., Gale, C. P., &amp; Johnson, O. A. (2018). Process mining in cardiology: A literature review. International Journal of Bioscience, Biochemistry and Bioinformatics, 8(4), 226–236. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.17706/ijbbb.2018.8.4.226</t>
+    </r>
   </si>
   <si>
     <t>“limitations in computer processing power, memory usage [...] and simplifying the control flow due to computational complexity”</t>
@@ -213,7 +315,7 @@
     <t>Computational resource constraints affect process mining</t>
   </si>
   <si>
-    <t>Business Process Model Retrieval Based on Graph Indexing Method</t>
+    <t>Rivas, D. F., Corchuelo, D. S., Figueroa, C., Corrales, J. C., &amp; Giugno, R. (2011). Business process model retrieval based on graph indexing method. In M. zur Muehlen &amp; J. Su (Eds.), Business process management workshops (pp. 238–250). Springer Berlin Heidelberg.</t>
   </si>
   <si>
     <t>“Many organizations with different degree of Business Process Management maturity have a considerable amount of business process models. Manage process collections inside an organization is a difficult task and demand many efforts to business analysts who need to expend time and knowledge taking important decisions. An example is introduced in [32] which use a repository containing about 500 process models to be consumed by local councils from Netherlands government. However, this number is small compared with thousands of processes that could have a multinational company. In this sense, an efficient system to manage and search for concrete and relevant processes is necessary.”</t>
@@ -222,6 +324,21 @@
     <t xml:space="preserve">Need efficient graph mining </t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Acheli, M., Grigori, D., &amp; Weidlich, M. (2019). Efficient discovery of compact maximal behavioral patterns from event logs. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/978-3-030-21290-2_36</t>
+    </r>
+  </si>
+  <si>
     <t>“Existing behavioral-pattern mining algorithms produce imprecise and redundant results, including non-maximal patterns that capture only part of frequent behavior and non-compact patterns that combine frequent and infrequent behavior; because these additional patterns provide no new process insights, discovery should retain only frequent, compact, maximal patterns that satisfy appropriate support and language-fitness criteria.”</t>
   </si>
   <si>
@@ -234,7 +351,19 @@
     <t>AI-enhanced pattern mining system should be able to rank and filter candidate patterns by relevance, for example rank the pattern by frequency and present top-N results, where N is a user configurable parameter, so that analysts can focus on the most relevant patterns while retaining access to rare and lower-ranked results.</t>
   </si>
   <si>
-    <t>Pattern Mining for Routine Behaviour Discovery in Pervasive Healthcare Environments</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Ali, R., ElHelw, M., Atallah, L., Lo, B., &amp; Yang, G.-Z. (2008). Pattern mining for routine behaviour discovery in pervasive healthcare environments. In 2008 International Conference on Information Technology and Applications in Biomedicine (pp. 241–244). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/ITAB.2008.4570576</t>
+    </r>
   </si>
   <si>
     <t>"Closed frequent pattern mining improves on this by limiting its search to patterns that are not subsets of any other pattern with the same support. This results in fewer redundant patterns"</t>
@@ -243,7 +372,7 @@
     <t>Redundant candidate patterns increase the pattern set</t>
   </si>
   <si>
-    <t>Approximate Data Mining Techniques on Clinical Data</t>
+    <t>Mantovani, M. (2020). Approximate data mining techniques on clinical data [Doctoral dissertation, University of Verona].</t>
   </si>
   <si>
     <t>“The number of rules it finds and outputs is often very large. This may hinder the discovery process and the interpretability of the results.”</t>
@@ -258,7 +387,19 @@
     <t>Struggles with complex BPMN structures</t>
   </si>
   <si>
-    <t>An Efficient Recommendation Method for Improving Business Process Modeling</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Li, Y., Cao, B., Xu, L., Yin, J., Deng, S., Yin, Y., &amp; Wu, Z. (2014). An efficient recommendation method for improving business process modeling. IEEE Transactions on Industrial Informatics, 10(1), 502–513. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/TII.2013.2258677</t>
+    </r>
   </si>
   <si>
     <t>"in this paper, we consider most basic structures except for iteration (loop) structures"</t>
@@ -276,7 +417,19 @@
     <t>" Meanwhile, since the iteration structure, which is not supported in our work, is common in business processes"</t>
   </si>
   <si>
-    <t>Discovering and Analyzing Contextual Behavioral</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Acheli, M., Grigori, D., &amp; Weidlich, M. (2022). Discovering and analyzing contextual behavioral patterns from event logs. IEEE Transactions on Knowledge and Data Engineering, 34(12), 5708–5721. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/TKDE.2021.3077653</t>
+    </r>
   </si>
   <si>
     <t>“The method, however, does not support loops and exclusive choices.”</t>
@@ -291,6 +444,21 @@
     <t>Implicit, approximate and non-contiguous pattern discovery</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Acheli, M., Grigori, D., &amp; Weidlich, M. (2019). Efficient discovery of compact maximal behavioral patterns from event logs. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/978-3-030-21290-2_36</t>
+    </r>
+  </si>
+  <si>
     <t>"Classical sequential pattern mining methods extract patterns corresponding to contiguous subsequences that occur in many sequences of a sequence database. No work has been done in the area to mine graphs that can contain arbitrary combinations of concur- rency, choices, sequential orderings, and loops in a single graph."</t>
   </si>
   <si>
@@ -303,12 +471,42 @@
     <t>AI-enhanced pattern mining system should be able to detect recurring patterns formed by activities that are not directly connected by sequence flows in the BPMN model., so that recurring behaviour is not missed when activities are separated by intermediate steps or complex control flow.</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Malhotra, K., Hobson, T. C., Valkova, S., Pullum, L. L., &amp; Ramanathan, A. (2015). Sequential pattern mining of electronic healthcare reimbursement claims: Experiences and challenges in uncovering how patients are treated by physicians. In 2015 IEEE International Conference on Big Data (Big Data) (pp. 2670–2679). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/BigData.2015.7364067</t>
+    </r>
+  </si>
+  <si>
     <t>“The drawback of this approach is that we do not capture concurrent occurrence of procedures.”</t>
   </si>
   <si>
     <t>Sequential representation fails to capture concurrency</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Perer, A., Wang, F., &amp; Hu, J. (2015). Mining and exploring care pathways from electronic medical records with visual analytics. Journal of Biomedical Informatics, 56, 369–378. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1016/j.jbi.2015.06.020</t>
+    </r>
+  </si>
+  <si>
     <t>“Such data characteristics yield a great challenge for frequent pattern mining algorithms, as they detect patterns with all possible combinations of events and subsets of events occurring at the same time. We refer to this phenomenon as pattern explosion.”</t>
   </si>
   <si>
@@ -321,7 +519,19 @@
     <t>Black-box nature of pattern mining</t>
   </si>
   <si>
-    <t>Analyzing Healthcare Processes with Incremental Process Discovery: Practical Insights from a Real-World Application</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Schuster, D., Benevento, E., Aloini, D., et al. (2024). Analyzing healthcare processes with incremental process discovery: Practical insights from a real-world application. Journal of Healthcare Informatics Research, 8, 523–554. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s41666-024-00165-6</t>
+    </r>
   </si>
   <si>
     <t>"Indeed, these approaches often produce so-called spaghetti models that are incomprehensible, challenging to interpret for healthcare managers, and of little informative value."</t>
@@ -348,12 +558,42 @@
     <t>Low interpretability and limited informative value</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Ali, R., ElHelw, M., Atallah, L., Lo, B., &amp; Yang, G.-Z. (2008). Pattern mining for routine behaviour discovery in pervasive healthcare environments. In 2008 International Conference on Information Technology and Applications in Biomedicine (pp. 241–244). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/ITAB.2008.4570576</t>
+    </r>
+  </si>
+  <si>
     <t>“While this is a powerful technique for general data streams, it is not an intuitive data structure for describing human routine.”</t>
   </si>
   <si>
     <t>Mined pattern representations are not intuitive</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Malhotra, K., Hobson, T. C., Valkova, S., Pullum, L. L., &amp; Ramanathan, A. (2015). Sequential pattern mining of electronic healthcare reimbursement claims: Experiences and challenges in uncovering how patients are treated by physicians. In 2015 IEEE International Conference on Big Data (Big Data) (pp. 2670–2679). </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1109/BigData.2015.7364067</t>
+    </r>
+  </si>
+  <si>
     <t>“Our study did not assign any meaning to the clinical procedure sequence patterns described here.”</t>
   </si>
   <si>
@@ -366,7 +606,19 @@
     <t>Automated quality-aware assessment</t>
   </si>
   <si>
-    <t>Split miner: automated discovery of accurate and simple business process models from event logs</t>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Augusto, A., Conforti, R., Dumas, M., La Rosa, M., &amp; Polyvyanyy, A. (2019). Split miner: Automated discovery of accurate and simple business process models from event logs. Knowledge and Information Systems, 59. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s10115-018-1214-x</t>
+    </r>
   </si>
   <si>
     <t>"striking a trade-off between these quality dimensions [fitness, precision, generalization, complexity] in a robust and scalable manner has proved elusive"</t>
@@ -381,7 +633,7 @@
     <t>AI-enhanced pattern mining system should automatically assess the quality of each discovered pattern against multiple quality dimensions (e.g., fitness, precision, generalization, complexity, and semantic meaningfulness) and present these quality metrics to the analyst to support informed decision-making and interpretation.</t>
   </si>
   <si>
-    <t>Evaluating the Comprehensibility of Control Flow Models Mined from the Sepsis Event Log</t>
+    <t>Zelefac, K. A. (2022). Evaluating the comprehensibility of control flow models mined from the sepsis event log [Master's thesis, Hasselt University].</t>
   </si>
   <si>
     <t>“They generate process models that do not find the right trade-off between simplicity, fitness, generalization, and precision.”</t>
@@ -390,6 +642,21 @@
     <t>Failure to balance multiple quality dimensions</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FFFFFFFF"/>
+      </rPr>
+      <t xml:space="preserve">Kusuma, G. P., Hall, M., Gale, C. P., &amp; Johnson, O. A. (2018). Process mining in cardiology: A literature review. International Journal of Bioscience, Biochemistry and Bioinformatics, 8(4), 226–236. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.17706/ijbbb.2018.8.4.226</t>
+    </r>
+  </si>
+  <si>
     <t>“bias associated with the mining algorithm”</t>
   </si>
   <si>
@@ -426,7 +693,19 @@
     <t>Frequent, rare, and anomalous pattern detection</t>
   </si>
   <si>
-    <t>Infrequent pattern mining in smart healthcare environment using data summarization</t>
+    <r>
+      <rPr>
+        <color rgb="FF1F1F1F"/>
+      </rPr>
+      <t xml:space="preserve">Ahmed, M., &amp; Barkat Ullah, A. S. S. M. (2018). Infrequent pattern mining in smart healthcare environment using data summarization. The Journal of Supercomputing, 74(10), 5041–5059. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s11227-018-2376-8</t>
+    </r>
   </si>
   <si>
     <t>"Existing summarization techniques create summaries which overlook the infrequent patterns such as anomalies in the data... As a result, the summaries include only a portion of the normal patterns of the data. In addition, when they are provided as input to anomaly detection algorithms... due to the absence of anomalies, computations become meaningless."</t>
@@ -435,6 +714,19 @@
     <t>Infrequent pattern are neglected and anomalies are omissioned</t>
   </si>
   <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">Acheli, M., Grigori, D., &amp; Weidlich, M. (2019). Efficient discovery of compact maximal behavioral patterns from event logs. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/978-3-030-21290-2_36</t>
+    </r>
+  </si>
+  <si>
     <t>"...and a comparatively high computational effort. That is, even though certain behavior is frequent, patterns may capture (i) only a part of the frequent behavior (i.e., they are not maximal), or (ii) a combination of frequent behavior with infrequent behavior (i.e., patterns are not compact)"</t>
   </si>
   <si>
@@ -459,7 +751,7 @@
     <t>Similarity, clustering, and process consolidation</t>
   </si>
   <si>
-    <t>Business Process Merging Based on Topic Cluster and Process Structure Matching</t>
+    <t>Huang, Y., &amp; You, I. (2016). Business process merging based on topic cluster and process structure matching. In K. Li, J. Li, Y. Liu, &amp; A. Castiglione (Eds.), Computational intelligence and intelligent systems (pp. 424–434). Springer Singapore.</t>
   </si>
   <si>
     <t>"similarities of activities to judge whether 2  processes can be consolidated"</t>
@@ -468,6 +760,19 @@
     <t>Activity similarity for process consolidation</t>
   </si>
   <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">Guo, C., &amp; Chen, J. (2019). Big data analytics in healthcare: Data-driven methods for typical treatment pattern mining. Journal of Systems Science and Systems Engineering, 28(6), 694–714. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s11518-019-5437-5</t>
+    </r>
+  </si>
+  <si>
     <t>"clustering large-scale treatment records is also a big challenge to extracting typical treatment patterns."</t>
   </si>
   <si>
@@ -478,6 +783,21 @@
   </si>
   <si>
     <t>Clustering evaluation uses accuracy and NMI</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <color rgb="FF1F1F1F"/>
+      </rPr>
+      <t xml:space="preserve">Ahmed, M., &amp; Barkat Ullah, A. S. S. M. (2018). Infrequent pattern mining in smart healthcare environment using data summarization. The Journal of Supercomputing, 74(10), 5041–5059. </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://doi.org/10.1007/s11227-018-2376-8</t>
+    </r>
   </si>
   <si>
     <t>" Clustering is the most important unsupervised machine learning technique, whose aim is to find natural or intrinsic groups of unlabelled objects... Using the concept of clustering, two different summary definitions have been widely used: centroid-based and feature-wise intersection-based summarization"</t>
@@ -508,7 +828,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="20">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -544,9 +864,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <strike/>
@@ -555,10 +885,54 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
       <b/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <color rgb="FF1F1F1F"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="38">
@@ -796,7 +1170,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="136">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -851,13 +1225,16 @@
     <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -866,7 +1243,7 @@
     <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -890,10 +1267,13 @@
     <xf borderId="0" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -945,13 +1325,16 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="14" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="11" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="15" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="15" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="16" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="16" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="17" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -966,7 +1349,7 @@
     <xf borderId="0" fillId="18" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="18" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="15" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -984,31 +1367,34 @@
     <xf borderId="1" fillId="17" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="18" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="18" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="18" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="18" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="18" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="18" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="18" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="18" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="18" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="16" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="19" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="19" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="20" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="20" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="21" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1032,10 +1418,13 @@
     <xf borderId="0" fillId="19" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="22" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="22" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="20" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="22" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="22" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="22" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1047,7 +1436,7 @@
     <xf borderId="0" fillId="23" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="24" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="24" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="25" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1071,7 +1460,7 @@
     <xf borderId="0" fillId="27" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="28" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="28" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="29" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1095,6 +1484,9 @@
     <xf borderId="0" fillId="27" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="28" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="30" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1107,7 +1499,7 @@
     <xf borderId="0" fillId="31" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="32" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="32" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="33" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -1125,6 +1517,9 @@
     <xf borderId="0" fillId="34" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="32" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="35" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1146,7 +1541,7 @@
     <xf borderId="0" fillId="36" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="36" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="36" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="36" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1158,6 +1553,9 @@
     <xf borderId="0" fillId="36" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="36" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="37" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1173,7 +1571,10 @@
     <xf borderId="0" fillId="37" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="37" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="37" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="37" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -1474,7 +1875,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="13.0"/>
     <col customWidth="1" min="2" max="2" width="37.75"/>
-    <col customWidth="1" min="3" max="3" width="47.25"/>
+    <col customWidth="1" min="3" max="3" width="71.13"/>
     <col customWidth="1" min="4" max="4" width="509.5"/>
     <col customWidth="1" min="5" max="5" width="97.38"/>
     <col customWidth="1" min="6" max="6" width="22.13"/>
@@ -1579,7 +1980,7 @@
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="13"/>
       <c r="B6" s="14"/>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="18" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="8" t="s">
@@ -1588,14 +1989,14 @@
       <c r="E6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="18"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="20"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="13"/>
       <c r="B7" s="14"/>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="18" t="s">
         <v>25</v>
       </c>
       <c r="D7" s="8" t="s">
@@ -1604,802 +2005,828 @@
       <c r="E7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="18"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="20"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="H8" s="28" t="s">
+      <c r="H8" s="29" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="29"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="23" t="s">
+      <c r="A9" s="30"/>
+      <c r="B9" s="31"/>
+      <c r="C9" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="31"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="35"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="29"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="23" t="s">
+      <c r="A10" s="30"/>
+      <c r="B10" s="31"/>
+      <c r="C10" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="38"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="29"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="23" t="s">
+      <c r="A11" s="30"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="37"/>
+      <c r="H11" s="38"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="39" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="40" t="s">
+      <c r="C12" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="41" t="s">
+      <c r="D12" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="42" t="s">
+      <c r="E12" s="43" t="s">
         <v>49</v>
       </c>
-      <c r="G12" s="43" t="s">
+      <c r="F12" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="H12" s="44" t="s">
+      <c r="G12" s="45" t="s">
         <v>51</v>
       </c>
+      <c r="H12" s="46" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="45"/>
-      <c r="B13" s="46"/>
-      <c r="C13" s="39" t="s">
+      <c r="A13" s="47"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="40" t="s">
+      <c r="D13" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="46"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="51"/>
+      <c r="K13" s="51"/>
+      <c r="L13" s="51"/>
+      <c r="M13" s="51"/>
+      <c r="N13" s="51"/>
+      <c r="O13" s="51"/>
+      <c r="P13" s="51"/>
+      <c r="Q13" s="51"/>
+      <c r="R13" s="51"/>
+      <c r="S13" s="51"/>
+      <c r="T13" s="51"/>
+      <c r="U13" s="51"/>
+      <c r="V13" s="51"/>
+      <c r="W13" s="51"/>
+      <c r="X13" s="51"/>
+      <c r="Y13" s="51"/>
+      <c r="Z13" s="51"/>
+      <c r="AA13" s="51"/>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="47"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="52" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="42" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="46"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="50"/>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="53" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="54" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="55" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="58" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" s="59" t="s">
+        <v>64</v>
+      </c>
+      <c r="H15" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="I15" s="51"/>
+      <c r="J15" s="51"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="51"/>
+      <c r="M15" s="51"/>
+      <c r="N15" s="51"/>
+      <c r="O15" s="51"/>
+      <c r="P15" s="51"/>
+      <c r="Q15" s="51"/>
+      <c r="R15" s="51"/>
+      <c r="S15" s="51"/>
+      <c r="T15" s="51"/>
+      <c r="U15" s="51"/>
+      <c r="V15" s="51"/>
+      <c r="W15" s="51"/>
+      <c r="X15" s="51"/>
+      <c r="Y15" s="51"/>
+      <c r="Z15" s="51"/>
+      <c r="AA15" s="51"/>
+      <c r="AB15" s="51"/>
+      <c r="AC15" s="51"/>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="53"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="55" t="s">
+        <v>65</v>
+      </c>
+      <c r="D16" s="56" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="57" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16" s="58"/>
+      <c r="G16" s="59"/>
+      <c r="H16" s="60"/>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="61"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="64" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="65" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="66"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="68"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="51"/>
+      <c r="L17" s="51"/>
+      <c r="M17" s="51"/>
+      <c r="N17" s="51"/>
+      <c r="O17" s="51"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="51"/>
+      <c r="R17" s="51"/>
+      <c r="S17" s="51"/>
+      <c r="T17" s="51"/>
+      <c r="U17" s="51"/>
+      <c r="V17" s="51"/>
+      <c r="W17" s="51"/>
+      <c r="X17" s="51"/>
+      <c r="Y17" s="51"/>
+      <c r="Z17" s="51"/>
+      <c r="AA17" s="51"/>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="61"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="55" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" s="56" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" s="57" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18" s="69" t="s">
+        <v>74</v>
+      </c>
+      <c r="G18" s="70" t="s">
+        <v>75</v>
+      </c>
+      <c r="H18" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" s="44"/>
-      <c r="G13" s="47"/>
-      <c r="H13" s="48"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
-      <c r="N13" s="49"/>
-      <c r="O13" s="49"/>
-      <c r="P13" s="49"/>
-      <c r="Q13" s="49"/>
-      <c r="R13" s="49"/>
-      <c r="S13" s="49"/>
-      <c r="T13" s="49"/>
-      <c r="U13" s="49"/>
-      <c r="V13" s="49"/>
-      <c r="W13" s="49"/>
-      <c r="X13" s="49"/>
-      <c r="Y13" s="49"/>
-      <c r="Z13" s="49"/>
-      <c r="AA13" s="49"/>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="45"/>
-      <c r="B14" s="46"/>
-      <c r="C14" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="D14" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E14" s="41" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="44"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="48"/>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="51" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15" s="52" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="53" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15" s="54" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="G15" s="56" t="s">
-        <v>62</v>
-      </c>
-      <c r="H15" s="57" t="s">
+      <c r="I18" s="51"/>
+      <c r="J18" s="51"/>
+      <c r="K18" s="51"/>
+      <c r="L18" s="51"/>
+      <c r="M18" s="51"/>
+      <c r="N18" s="51"/>
+      <c r="O18" s="51"/>
+      <c r="P18" s="51"/>
+      <c r="Q18" s="51"/>
+      <c r="R18" s="51"/>
+      <c r="S18" s="51"/>
+      <c r="T18" s="51"/>
+      <c r="U18" s="51"/>
+      <c r="V18" s="51"/>
+      <c r="W18" s="51"/>
+      <c r="X18" s="51"/>
+      <c r="Y18" s="51"/>
+      <c r="Z18" s="51"/>
+      <c r="AA18" s="51"/>
+      <c r="AB18" s="51"/>
+      <c r="AC18" s="51"/>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="61"/>
+      <c r="B19" s="62"/>
+      <c r="C19" s="55" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="56" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="57" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="69"/>
+      <c r="G19" s="70"/>
+      <c r="H19" s="71"/>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="61"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="72" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="56" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="57" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" s="69"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="71"/>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="73" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="74" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="75" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" s="76" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" s="77" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" s="78" t="s">
+        <v>87</v>
+      </c>
+      <c r="G21" s="79" t="s">
+        <v>88</v>
+      </c>
+      <c r="H21" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="I15" s="49"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="49"/>
-      <c r="L15" s="49"/>
-      <c r="M15" s="49"/>
-      <c r="N15" s="49"/>
-      <c r="O15" s="49"/>
-      <c r="P15" s="49"/>
-      <c r="Q15" s="49"/>
-      <c r="R15" s="49"/>
-      <c r="S15" s="49"/>
-      <c r="T15" s="49"/>
-      <c r="U15" s="49"/>
-      <c r="V15" s="49"/>
-      <c r="W15" s="49"/>
-      <c r="X15" s="49"/>
-      <c r="Y15" s="49"/>
-      <c r="Z15" s="49"/>
-      <c r="AA15" s="49"/>
-      <c r="AB15" s="49"/>
-      <c r="AC15" s="49"/>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="50"/>
-      <c r="B16" s="51"/>
-      <c r="C16" s="52" t="s">
-        <v>63</v>
-      </c>
-      <c r="D16" s="53" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" s="54" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="55"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="57"/>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="58"/>
-      <c r="B17" s="59"/>
-      <c r="C17" s="60" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="61" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="62" t="s">
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="81"/>
+      <c r="B22" s="82"/>
+      <c r="C22" s="83"/>
+      <c r="D22" s="76" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="77" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="84"/>
+      <c r="G22" s="85"/>
+      <c r="H22" s="86"/>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="81"/>
+      <c r="B23" s="82"/>
+      <c r="C23" s="75" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="76" t="s">
+        <v>91</v>
+      </c>
+      <c r="E23" s="77" t="s">
+        <v>92</v>
+      </c>
+      <c r="F23" s="84"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="86"/>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="87" t="s">
+        <v>93</v>
+      </c>
+      <c r="B24" s="88" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="89" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" s="90" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="91" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" s="92" t="s">
+        <v>98</v>
+      </c>
+      <c r="G24" s="93" t="s">
+        <v>99</v>
+      </c>
+      <c r="H24" s="94" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="87"/>
+      <c r="B25" s="88"/>
+      <c r="C25" s="89" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" s="90" t="s">
+        <v>101</v>
+      </c>
+      <c r="E25" s="91" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="92"/>
+      <c r="G25" s="93"/>
+      <c r="H25" s="94"/>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="87"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="89" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="90" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" s="91" t="s">
+        <v>105</v>
+      </c>
+      <c r="F26" s="92"/>
+      <c r="G26" s="93"/>
+      <c r="H26" s="94"/>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="95" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" s="96" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="97" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="98" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="99" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="G27" s="101" t="s">
+        <v>112</v>
+      </c>
+      <c r="H27" s="102" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="103"/>
+      <c r="B28" s="104"/>
+      <c r="C28" s="105"/>
+      <c r="D28" s="98" t="s">
+        <v>113</v>
+      </c>
+      <c r="E28" s="99" t="s">
+        <v>114</v>
+      </c>
+      <c r="F28" s="102"/>
+      <c r="G28" s="106"/>
+      <c r="H28" s="107"/>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="103"/>
+      <c r="B29" s="104"/>
+      <c r="C29" s="105"/>
+      <c r="D29" s="98" t="s">
+        <v>115</v>
+      </c>
+      <c r="E29" s="99" t="s">
+        <v>116</v>
+      </c>
+      <c r="F29" s="102"/>
+      <c r="G29" s="106"/>
+      <c r="H29" s="107"/>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="103"/>
+      <c r="B30" s="104"/>
+      <c r="C30" s="97" t="s">
+        <v>117</v>
+      </c>
+      <c r="D30" s="98" t="s">
+        <v>118</v>
+      </c>
+      <c r="E30" s="99" t="s">
+        <v>119</v>
+      </c>
+      <c r="F30" s="102"/>
+      <c r="G30" s="106"/>
+      <c r="H30" s="107"/>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="103"/>
+      <c r="B31" s="104"/>
+      <c r="C31" s="97" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" s="98" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" s="99" t="s">
+        <v>122</v>
+      </c>
+      <c r="F31" s="102"/>
+      <c r="G31" s="106"/>
+      <c r="H31" s="107"/>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="108" t="s">
+        <v>123</v>
+      </c>
+      <c r="B32" s="109" t="s">
+        <v>124</v>
+      </c>
+      <c r="C32" s="110" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" s="111" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="112" t="s">
+        <v>127</v>
+      </c>
+      <c r="F32" s="113" t="s">
+        <v>128</v>
+      </c>
+      <c r="G32" s="114" t="s">
+        <v>129</v>
+      </c>
+      <c r="H32" s="115" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="108"/>
+      <c r="B33" s="109"/>
+      <c r="C33" s="116" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="111" t="s">
+        <v>131</v>
+      </c>
+      <c r="E33" s="112" t="s">
+        <v>132</v>
+      </c>
+      <c r="F33" s="113"/>
+      <c r="G33" s="114"/>
+      <c r="H33" s="115"/>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="108"/>
+      <c r="B34" s="109"/>
+      <c r="C34" s="110" t="s">
+        <v>133</v>
+      </c>
+      <c r="D34" s="111" t="s">
+        <v>134</v>
+      </c>
+      <c r="E34" s="112" t="s">
+        <v>135</v>
+      </c>
+      <c r="F34" s="113"/>
+      <c r="G34" s="114"/>
+      <c r="H34" s="115"/>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="118" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="118" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="63"/>
-      <c r="G17" s="64"/>
-      <c r="H17" s="65"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="49"/>
-      <c r="L17" s="49"/>
-      <c r="M17" s="49"/>
-      <c r="N17" s="49"/>
-      <c r="O17" s="49"/>
-      <c r="P17" s="49"/>
-      <c r="Q17" s="49"/>
-      <c r="R17" s="49"/>
-      <c r="S17" s="49"/>
-      <c r="T17" s="49"/>
-      <c r="U17" s="49"/>
-      <c r="V17" s="49"/>
-      <c r="W17" s="49"/>
-      <c r="X17" s="49"/>
-      <c r="Y17" s="49"/>
-      <c r="Z17" s="49"/>
-      <c r="AA17" s="49"/>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="58"/>
-      <c r="B18" s="59"/>
-      <c r="C18" s="52" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="53" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" s="54" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="66" t="s">
-        <v>71</v>
-      </c>
-      <c r="G18" s="67" t="s">
-        <v>72</v>
-      </c>
-      <c r="H18" s="68" t="s">
-        <v>51</v>
-      </c>
-      <c r="I18" s="49"/>
-      <c r="J18" s="49"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="49"/>
-      <c r="N18" s="49"/>
-      <c r="O18" s="49"/>
-      <c r="P18" s="49"/>
-      <c r="Q18" s="49"/>
-      <c r="R18" s="49"/>
-      <c r="S18" s="49"/>
-      <c r="T18" s="49"/>
-      <c r="U18" s="49"/>
-      <c r="V18" s="49"/>
-      <c r="W18" s="49"/>
-      <c r="X18" s="49"/>
-      <c r="Y18" s="49"/>
-      <c r="Z18" s="49"/>
-      <c r="AA18" s="49"/>
-      <c r="AB18" s="49"/>
-      <c r="AC18" s="49"/>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="58"/>
-      <c r="B19" s="59"/>
-      <c r="C19" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="D19" s="53" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" s="54" t="s">
-        <v>75</v>
-      </c>
-      <c r="F19" s="66"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="68"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="58"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="52" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="F20" s="66"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="68"/>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="69" t="s">
-        <v>79</v>
-      </c>
-      <c r="B21" s="70" t="s">
-        <v>80</v>
-      </c>
-      <c r="C21" s="71" t="s">
-        <v>81</v>
-      </c>
-      <c r="D21" s="72" t="s">
-        <v>82</v>
-      </c>
-      <c r="E21" s="73" t="s">
-        <v>83</v>
-      </c>
-      <c r="F21" s="74" t="s">
-        <v>84</v>
-      </c>
-      <c r="G21" s="75" t="s">
-        <v>85</v>
-      </c>
-      <c r="H21" s="76" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="77"/>
-      <c r="B22" s="78"/>
-      <c r="C22" s="71"/>
-      <c r="D22" s="72" t="s">
-        <v>86</v>
-      </c>
-      <c r="E22" s="73" t="s">
-        <v>83</v>
-      </c>
-      <c r="F22" s="79"/>
-      <c r="G22" s="80"/>
-      <c r="H22" s="81"/>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="77"/>
-      <c r="B23" s="78"/>
-      <c r="C23" s="71" t="s">
-        <v>87</v>
-      </c>
-      <c r="D23" s="72" t="s">
-        <v>88</v>
-      </c>
-      <c r="E23" s="73" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="79"/>
-      <c r="G23" s="80"/>
-      <c r="H23" s="81"/>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="82" t="s">
-        <v>90</v>
-      </c>
-      <c r="B24" s="83" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24" s="84" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="85" t="s">
-        <v>92</v>
-      </c>
-      <c r="E24" s="86" t="s">
-        <v>93</v>
-      </c>
-      <c r="F24" s="87" t="s">
-        <v>94</v>
-      </c>
-      <c r="G24" s="88" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="89" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="82"/>
-      <c r="B25" s="83"/>
-      <c r="C25" s="84" t="s">
-        <v>54</v>
-      </c>
-      <c r="D25" s="85" t="s">
-        <v>96</v>
-      </c>
-      <c r="E25" s="86" t="s">
-        <v>97</v>
-      </c>
-      <c r="F25" s="87"/>
-      <c r="G25" s="88"/>
-      <c r="H25" s="89"/>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="82"/>
-      <c r="B26" s="83"/>
-      <c r="C26" s="84" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="85" t="s">
-        <v>98</v>
-      </c>
-      <c r="E26" s="86" t="s">
-        <v>99</v>
-      </c>
-      <c r="F26" s="87"/>
-      <c r="G26" s="88"/>
-      <c r="H26" s="89"/>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="90" t="s">
-        <v>100</v>
-      </c>
-      <c r="B27" s="91" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" s="92" t="s">
-        <v>102</v>
-      </c>
-      <c r="D27" s="93" t="s">
-        <v>103</v>
-      </c>
-      <c r="E27" s="94" t="s">
-        <v>104</v>
-      </c>
-      <c r="F27" s="95" t="s">
-        <v>105</v>
-      </c>
-      <c r="G27" s="96" t="s">
-        <v>106</v>
-      </c>
-      <c r="H27" s="97" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="98"/>
-      <c r="B28" s="99"/>
-      <c r="C28" s="92"/>
-      <c r="D28" s="93" t="s">
-        <v>107</v>
-      </c>
-      <c r="E28" s="94" t="s">
-        <v>108</v>
-      </c>
-      <c r="F28" s="97"/>
-      <c r="G28" s="100"/>
-      <c r="H28" s="101"/>
-    </row>
-    <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="98"/>
-      <c r="B29" s="99"/>
-      <c r="C29" s="92"/>
-      <c r="D29" s="93" t="s">
-        <v>109</v>
-      </c>
-      <c r="E29" s="94" t="s">
-        <v>110</v>
-      </c>
-      <c r="F29" s="97"/>
-      <c r="G29" s="100"/>
-      <c r="H29" s="101"/>
-    </row>
-    <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="98"/>
-      <c r="B30" s="99"/>
-      <c r="C30" s="92" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" s="93" t="s">
-        <v>111</v>
-      </c>
-      <c r="E30" s="94" t="s">
-        <v>112</v>
-      </c>
-      <c r="F30" s="97"/>
-      <c r="G30" s="100"/>
-      <c r="H30" s="101"/>
-    </row>
-    <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="98"/>
-      <c r="B31" s="99"/>
-      <c r="C31" s="92" t="s">
-        <v>54</v>
-      </c>
-      <c r="D31" s="93" t="s">
-        <v>113</v>
-      </c>
-      <c r="E31" s="94" t="s">
-        <v>114</v>
-      </c>
-      <c r="F31" s="97"/>
-      <c r="G31" s="100"/>
-      <c r="H31" s="101"/>
-    </row>
-    <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="102" t="s">
-        <v>115</v>
-      </c>
-      <c r="B32" s="103" t="s">
-        <v>116</v>
-      </c>
-      <c r="C32" s="104" t="s">
-        <v>117</v>
-      </c>
-      <c r="D32" s="105" t="s">
-        <v>118</v>
-      </c>
-      <c r="E32" s="106" t="s">
-        <v>119</v>
-      </c>
-      <c r="F32" s="107" t="s">
-        <v>120</v>
-      </c>
-      <c r="G32" s="108" t="s">
-        <v>121</v>
-      </c>
-      <c r="H32" s="109" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="102"/>
-      <c r="B33" s="103"/>
-      <c r="C33" s="104" t="s">
-        <v>122</v>
-      </c>
-      <c r="D33" s="105" t="s">
-        <v>123</v>
-      </c>
-      <c r="E33" s="106" t="s">
-        <v>124</v>
-      </c>
-      <c r="F33" s="107"/>
-      <c r="G33" s="108"/>
-      <c r="H33" s="109"/>
-    </row>
-    <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="102"/>
-      <c r="B34" s="103"/>
-      <c r="C34" s="104" t="s">
-        <v>63</v>
-      </c>
-      <c r="D34" s="105" t="s">
-        <v>125</v>
-      </c>
-      <c r="E34" s="106" t="s">
-        <v>126</v>
-      </c>
-      <c r="F34" s="107"/>
-      <c r="G34" s="108"/>
-      <c r="H34" s="109"/>
-    </row>
-    <row r="35" ht="22.5" customHeight="1">
-      <c r="A35" s="110" t="s">
-        <v>127</v>
-      </c>
-      <c r="B35" s="111" t="s">
-        <v>128</v>
-      </c>
-      <c r="C35" s="111" t="s">
-        <v>66</v>
-      </c>
-      <c r="D35" s="112" t="s">
-        <v>129</v>
-      </c>
-      <c r="E35" s="111" t="s">
-        <v>130</v>
-      </c>
-      <c r="F35" s="113"/>
-      <c r="G35" s="114"/>
-      <c r="H35" s="110"/>
+      <c r="D35" s="119" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" s="118" t="s">
+        <v>139</v>
+      </c>
+      <c r="F35" s="120"/>
+      <c r="G35" s="121"/>
+      <c r="H35" s="117"/>
     </row>
     <row r="36" ht="22.5" customHeight="1">
-      <c r="A36" s="110"/>
-      <c r="B36" s="111"/>
-      <c r="C36" s="111"/>
-      <c r="D36" s="112" t="s">
-        <v>131</v>
-      </c>
-      <c r="E36" s="111" t="s">
-        <v>132</v>
-      </c>
-      <c r="F36" s="113"/>
-      <c r="G36" s="114"/>
-      <c r="H36" s="110"/>
+      <c r="A36" s="117"/>
+      <c r="B36" s="118"/>
+      <c r="C36" s="118"/>
+      <c r="D36" s="119" t="s">
+        <v>140</v>
+      </c>
+      <c r="E36" s="118" t="s">
+        <v>141</v>
+      </c>
+      <c r="F36" s="120"/>
+      <c r="G36" s="121"/>
+      <c r="H36" s="117"/>
     </row>
     <row r="37" ht="22.5" customHeight="1">
-      <c r="A37" s="110"/>
-      <c r="B37" s="111"/>
-      <c r="C37" s="111" t="s">
+      <c r="A37" s="117"/>
+      <c r="B37" s="118"/>
+      <c r="C37" s="118" t="s">
         <v>36</v>
       </c>
-      <c r="D37" s="112" t="s">
-        <v>133</v>
-      </c>
-      <c r="E37" s="111" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="113"/>
-      <c r="G37" s="114"/>
-      <c r="H37" s="110"/>
+      <c r="D37" s="119" t="s">
+        <v>142</v>
+      </c>
+      <c r="E37" s="118" t="s">
+        <v>143</v>
+      </c>
+      <c r="F37" s="120"/>
+      <c r="G37" s="121"/>
+      <c r="H37" s="117"/>
     </row>
     <row r="38" ht="22.5" customHeight="1">
-      <c r="A38" s="115" t="s">
-        <v>135</v>
-      </c>
-      <c r="B38" s="116" t="s">
-        <v>136</v>
-      </c>
-      <c r="C38" s="117" t="s">
-        <v>137</v>
-      </c>
-      <c r="D38" s="118" t="s">
-        <v>138</v>
-      </c>
-      <c r="E38" s="116" t="s">
-        <v>139</v>
-      </c>
-      <c r="F38" s="119"/>
-      <c r="G38" s="120"/>
-      <c r="H38" s="115"/>
+      <c r="A38" s="122" t="s">
+        <v>144</v>
+      </c>
+      <c r="B38" s="123" t="s">
+        <v>145</v>
+      </c>
+      <c r="C38" s="124" t="s">
+        <v>146</v>
+      </c>
+      <c r="D38" s="125" t="s">
+        <v>147</v>
+      </c>
+      <c r="E38" s="123" t="s">
+        <v>148</v>
+      </c>
+      <c r="F38" s="126"/>
+      <c r="G38" s="127"/>
+      <c r="H38" s="122"/>
     </row>
     <row r="39" ht="22.5" customHeight="1">
-      <c r="A39" s="115"/>
-      <c r="B39" s="116"/>
-      <c r="C39" s="116" t="s">
-        <v>22</v>
-      </c>
-      <c r="D39" s="118" t="s">
-        <v>140</v>
-      </c>
-      <c r="E39" s="116" t="s">
-        <v>141</v>
-      </c>
-      <c r="F39" s="119"/>
-      <c r="G39" s="120"/>
-      <c r="H39" s="115"/>
+      <c r="A39" s="122"/>
+      <c r="B39" s="123"/>
+      <c r="C39" s="128" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" s="125" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" s="123" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" s="126"/>
+      <c r="G39" s="127"/>
+      <c r="H39" s="122"/>
     </row>
     <row r="40" ht="22.5" customHeight="1">
-      <c r="A40" s="110" t="s">
-        <v>142</v>
-      </c>
-      <c r="B40" s="111" t="s">
-        <v>143</v>
-      </c>
-      <c r="C40" s="111" t="s">
-        <v>30</v>
-      </c>
-      <c r="D40" s="112" t="s">
-        <v>144</v>
-      </c>
-      <c r="E40" s="111" t="s">
-        <v>145</v>
-      </c>
-      <c r="F40" s="113"/>
-      <c r="G40" s="114"/>
-      <c r="H40" s="110"/>
+      <c r="A40" s="117" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" s="118" t="s">
+        <v>153</v>
+      </c>
+      <c r="C40" s="118" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="119" t="s">
+        <v>154</v>
+      </c>
+      <c r="E40" s="118" t="s">
+        <v>155</v>
+      </c>
+      <c r="F40" s="120"/>
+      <c r="G40" s="121"/>
+      <c r="H40" s="117"/>
     </row>
     <row r="41" ht="22.5" customHeight="1">
-      <c r="A41" s="121" t="s">
-        <v>146</v>
-      </c>
-      <c r="B41" s="122" t="s">
-        <v>147</v>
-      </c>
-      <c r="C41" s="122" t="s">
-        <v>148</v>
-      </c>
-      <c r="D41" s="123" t="s">
-        <v>149</v>
-      </c>
-      <c r="E41" s="122" t="s">
-        <v>150</v>
-      </c>
-      <c r="F41" s="124"/>
-      <c r="G41" s="125"/>
-      <c r="H41" s="121"/>
+      <c r="A41" s="129" t="s">
+        <v>156</v>
+      </c>
+      <c r="B41" s="130" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="130" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" s="131" t="s">
+        <v>159</v>
+      </c>
+      <c r="E41" s="130" t="s">
+        <v>160</v>
+      </c>
+      <c r="F41" s="132"/>
+      <c r="G41" s="133"/>
+      <c r="H41" s="129"/>
     </row>
     <row r="42" ht="22.5" customHeight="1">
-      <c r="A42" s="121"/>
-      <c r="B42" s="122"/>
-      <c r="C42" s="122" t="s">
-        <v>30</v>
-      </c>
-      <c r="D42" s="123" t="s">
-        <v>151</v>
-      </c>
-      <c r="E42" s="122" t="s">
-        <v>152</v>
-      </c>
-      <c r="F42" s="124"/>
-      <c r="G42" s="125"/>
-      <c r="H42" s="121"/>
+      <c r="A42" s="129"/>
+      <c r="B42" s="130"/>
+      <c r="C42" s="134" t="s">
+        <v>161</v>
+      </c>
+      <c r="D42" s="131" t="s">
+        <v>162</v>
+      </c>
+      <c r="E42" s="130" t="s">
+        <v>163</v>
+      </c>
+      <c r="F42" s="132"/>
+      <c r="G42" s="133"/>
+      <c r="H42" s="129"/>
     </row>
     <row r="43" ht="22.5" customHeight="1">
-      <c r="A43" s="121"/>
-      <c r="B43" s="122"/>
-      <c r="C43" s="122"/>
-      <c r="D43" s="123" t="s">
-        <v>153</v>
-      </c>
-      <c r="E43" s="122" t="s">
-        <v>154</v>
-      </c>
-      <c r="F43" s="124"/>
-      <c r="G43" s="125"/>
-      <c r="H43" s="121"/>
+      <c r="A43" s="129"/>
+      <c r="B43" s="130"/>
+      <c r="C43" s="130"/>
+      <c r="D43" s="131" t="s">
+        <v>164</v>
+      </c>
+      <c r="E43" s="130" t="s">
+        <v>165</v>
+      </c>
+      <c r="F43" s="132"/>
+      <c r="G43" s="133"/>
+      <c r="H43" s="129"/>
     </row>
     <row r="44" ht="22.5" customHeight="1">
-      <c r="A44" s="121"/>
-      <c r="B44" s="122"/>
-      <c r="C44" s="126" t="s">
-        <v>137</v>
-      </c>
-      <c r="D44" s="123" t="s">
-        <v>155</v>
-      </c>
-      <c r="E44" s="122" t="s">
-        <v>156</v>
-      </c>
-      <c r="F44" s="124"/>
-      <c r="G44" s="125"/>
-      <c r="H44" s="121"/>
+      <c r="A44" s="129"/>
+      <c r="B44" s="130"/>
+      <c r="C44" s="135" t="s">
+        <v>166</v>
+      </c>
+      <c r="D44" s="131" t="s">
+        <v>167</v>
+      </c>
+      <c r="E44" s="130" t="s">
+        <v>168</v>
+      </c>
+      <c r="F44" s="132"/>
+      <c r="G44" s="133"/>
+      <c r="H44" s="129"/>
     </row>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="110" t="s">
-        <v>157</v>
-      </c>
-      <c r="B45" s="111" t="s">
+      <c r="A45" s="117" t="s">
+        <v>169</v>
+      </c>
+      <c r="B45" s="118" t="s">
+        <v>170</v>
+      </c>
+      <c r="C45" s="118" t="s">
         <v>158</v>
       </c>
-      <c r="C45" s="111" t="s">
-        <v>148</v>
-      </c>
-      <c r="D45" s="112" t="s">
-        <v>159</v>
-      </c>
-      <c r="E45" s="111" t="s">
-        <v>160</v>
-      </c>
-      <c r="F45" s="113"/>
-      <c r="G45" s="114"/>
-      <c r="H45" s="110"/>
+      <c r="D45" s="119" t="s">
+        <v>171</v>
+      </c>
+      <c r="E45" s="118" t="s">
+        <v>172</v>
+      </c>
+      <c r="F45" s="120"/>
+      <c r="G45" s="121"/>
+      <c r="H45" s="117"/>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="110"/>
-      <c r="B46" s="111"/>
-      <c r="C46" s="111"/>
-      <c r="D46" s="112" t="s">
-        <v>161</v>
-      </c>
-      <c r="E46" s="111" t="s">
-        <v>162</v>
-      </c>
-      <c r="F46" s="113"/>
-      <c r="G46" s="114"/>
-      <c r="H46" s="110"/>
+      <c r="A46" s="117"/>
+      <c r="B46" s="118"/>
+      <c r="C46" s="118"/>
+      <c r="D46" s="119" t="s">
+        <v>173</v>
+      </c>
+      <c r="E46" s="118" t="s">
+        <v>174</v>
+      </c>
+      <c r="F46" s="120"/>
+      <c r="G46" s="121"/>
+      <c r="H46" s="117"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="C6"/>
+    <hyperlink r:id="rId2" ref="C7"/>
+    <hyperlink r:id="rId3" ref="C8"/>
+    <hyperlink r:id="rId4" ref="C10"/>
+    <hyperlink r:id="rId5" ref="C11"/>
+    <hyperlink r:id="rId6" ref="C14"/>
+    <hyperlink r:id="rId7" ref="C15"/>
+    <hyperlink r:id="rId8" ref="C16"/>
+    <hyperlink r:id="rId9" ref="C18"/>
+    <hyperlink r:id="rId10" ref="C19"/>
+    <hyperlink r:id="rId11" ref="C21"/>
+    <hyperlink r:id="rId12" ref="C23"/>
+    <hyperlink r:id="rId13" ref="C24"/>
+    <hyperlink r:id="rId14" ref="C25"/>
+    <hyperlink r:id="rId15" ref="C26"/>
+    <hyperlink r:id="rId16" ref="C27"/>
+    <hyperlink r:id="rId17" ref="C30"/>
+    <hyperlink r:id="rId18" ref="C31"/>
+    <hyperlink r:id="rId19" ref="C32"/>
+    <hyperlink r:id="rId20" ref="C34"/>
+    <hyperlink r:id="rId21" ref="C38"/>
+    <hyperlink r:id="rId22" ref="C39"/>
+    <hyperlink r:id="rId23" ref="C42"/>
+    <hyperlink r:id="rId24" ref="C44"/>
+  </hyperlinks>
+  <drawing r:id="rId25"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId27"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>